<commit_message>
fixed run issue in encoding and retrieval, enlargened image size
</commit_message>
<xml_diff>
--- a/retrieval_task_behav/runs_params.xlsx
+++ b/retrieval_task_behav/runs_params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nitzanlubi/My Drive/Lab/schema_based_learning/retrieval_exp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviayin/Desktop/sbl_realistic integration/retrieval_task_behav/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F73FA1-00CF-DC4D-91C1-AB54D3F7802E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189738FA-7BBC-7549-90B9-ABCE2DEC2546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="28800" windowHeight="17500" xr2:uid="{1EB1B345-0735-2F41-AEFE-886AE22BCD6A}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="17260" xr2:uid="{1EB1B345-0735-2F41-AEFE-886AE22BCD6A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -393,7 +393,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC6E2131-7787-1E47-9E97-F45B950C3EB9}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -403,26 +403,21 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>3</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Changes made with Nitzan: fixing retrieval and encoding image size, fixing to four runs for retrieval, etc.
</commit_message>
<xml_diff>
--- a/retrieval_task_behav/runs_params.xlsx
+++ b/retrieval_task_behav/runs_params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliviayin/Desktop/sbl_realistic integration/retrieval_task_behav/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\nitzan\SBL\sbl_integration_May_29\retrieval_task_behav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189738FA-7BBC-7549-90B9-ABCE2DEC2546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{445C097B-0DAE-4900-8131-D88B8CE0ECE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="17260" xr2:uid="{1EB1B345-0735-2F41-AEFE-886AE22BCD6A}"/>
+    <workbookView xWindow="4815" yWindow="3525" windowWidth="10920" windowHeight="14520" xr2:uid="{1EB1B345-0735-2F41-AEFE-886AE22BCD6A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -393,31 +393,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC6E2131-7787-1E47-9E97-F45B950C3EB9}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>3</v>
       </c>
-      <c r="B4" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>